<commit_message>
Added: status column  applicant internal service template
</commit_message>
<xml_diff>
--- a/storage/app/template/applicantInternalService.xlsx
+++ b/storage/app/template/applicantInternalService.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Project\RSP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E2EF3D9-380C-4172-9A38-FF4B7F67B709}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB9B49D8-0376-41FD-843C-D134FEAD329C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{8113A99E-9156-40D8-A2D8-36A56E68640F}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
     <t xml:space="preserve">PUBLICATION DATE: </t>
   </si>
@@ -73,6 +73,9 @@
   <si>
     <t>SALARY 
 GRADE</t>
+  </si>
+  <si>
+    <t>STATUS</t>
   </si>
 </sst>
 </file>
@@ -488,24 +491,24 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A02B2E2A-17B3-4664-9767-1B738A9DDE6E}">
-  <dimension ref="A1:K8"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.28515625" style="1" customWidth="1"/>
     <col min="2" max="2" width="4.5703125" style="2" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="42.28515625" style="2" customWidth="1"/>
-    <col min="4" max="4" width="13.28515625" style="1" customWidth="1"/>
-    <col min="5" max="5" width="22.28515625" style="1" customWidth="1"/>
-    <col min="6" max="6" width="13" style="1" customWidth="1"/>
-    <col min="7" max="7" width="15" style="1" customWidth="1"/>
-    <col min="8" max="8" width="14.5703125" style="1" customWidth="1"/>
-    <col min="9" max="9" width="39.28515625" style="2" customWidth="1"/>
-    <col min="10" max="10" width="19.140625" style="1" customWidth="1"/>
-    <col min="11" max="11" width="13.42578125" style="1" customWidth="1"/>
-    <col min="12" max="16384" width="9.140625" style="7"/>
+    <col min="4" max="5" width="13.140625" style="1" customWidth="1"/>
+    <col min="6" max="6" width="22.28515625" style="1" customWidth="1"/>
+    <col min="7" max="7" width="13" style="1" customWidth="1"/>
+    <col min="8" max="8" width="15" style="1" customWidth="1"/>
+    <col min="9" max="9" width="14.5703125" style="1" customWidth="1"/>
+    <col min="10" max="10" width="39.28515625" style="2" customWidth="1"/>
+    <col min="11" max="11" width="19.140625" style="1" customWidth="1"/>
+    <col min="12" max="12" width="13.42578125" style="1" customWidth="1"/>
+    <col min="13" max="16384" width="9.140625" style="7"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" s="3"/>
       <c r="B1" s="4"/>
       <c r="C1" s="4"/>
@@ -514,11 +517,12 @@
       <c r="F1" s="3"/>
       <c r="G1" s="3"/>
       <c r="H1" s="3"/>
-      <c r="I1" s="4"/>
-      <c r="J1" s="3"/>
+      <c r="I1" s="3"/>
+      <c r="J1" s="4"/>
       <c r="K1" s="3"/>
+      <c r="L1" s="3"/>
     </row>
-    <row r="2" spans="1:11" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:12" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
         <v>2</v>
       </c>
@@ -527,13 +531,14 @@
       <c r="D2" s="10"/>
       <c r="E2" s="10"/>
       <c r="F2" s="10"/>
-      <c r="G2" s="8"/>
+      <c r="G2" s="10"/>
       <c r="H2" s="8"/>
       <c r="I2" s="8"/>
       <c r="J2" s="8"/>
       <c r="K2" s="8"/>
+      <c r="L2" s="8"/>
     </row>
-    <row r="3" spans="1:11" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:12" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
         <v>0</v>
       </c>
@@ -542,13 +547,14 @@
       <c r="D3" s="10"/>
       <c r="E3" s="10"/>
       <c r="F3" s="10"/>
-      <c r="G3" s="9"/>
+      <c r="G3" s="10"/>
       <c r="H3" s="9"/>
       <c r="I3" s="9"/>
       <c r="J3" s="9"/>
       <c r="K3" s="9"/>
+      <c r="L3" s="9"/>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" s="3"/>
       <c r="B4" s="4"/>
       <c r="C4" s="4"/>
@@ -557,11 +563,12 @@
       <c r="F4" s="3"/>
       <c r="G4" s="3"/>
       <c r="H4" s="3"/>
-      <c r="I4" s="4"/>
-      <c r="J4" s="3"/>
+      <c r="I4" s="3"/>
+      <c r="J4" s="4"/>
       <c r="K4" s="3"/>
+      <c r="L4" s="3"/>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" s="3"/>
       <c r="B5" s="4"/>
       <c r="C5" s="4"/>
@@ -570,11 +577,12 @@
       <c r="F5" s="3"/>
       <c r="G5" s="3"/>
       <c r="H5" s="3"/>
-      <c r="I5" s="4"/>
-      <c r="J5" s="3"/>
+      <c r="I5" s="3"/>
+      <c r="J5" s="4"/>
       <c r="K5" s="3"/>
+      <c r="L5" s="3"/>
     </row>
-    <row r="6" spans="1:11" ht="27" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:12" ht="27" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
         <v>3</v>
       </c>
@@ -588,26 +596,29 @@
         <v>5</v>
       </c>
       <c r="E6" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="F6" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="F6" s="5" t="s">
+      <c r="G6" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="G6" s="5" t="s">
+      <c r="H6" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="H6" s="5" t="s">
+      <c r="I6" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="I6" s="5" t="s">
+      <c r="J6" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="J6" s="5" t="s">
+      <c r="K6" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="K6" s="7"/>
+      <c r="L6" s="7"/>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8" s="6"/>
       <c r="B8" s="6"/>
       <c r="C8" s="6"/>
@@ -619,11 +630,12 @@
       <c r="I8" s="6"/>
       <c r="J8" s="6"/>
       <c r="K8" s="6"/>
+      <c r="L8" s="6"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A3:F3"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A3:G3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>

</xml_diff>